<commit_message>
Experimental procedure v2 - 2026_07_15 - ksweep
</commit_message>
<xml_diff>
--- a/publication/2026_07_10_results_xp_all_datasets_phd_contribution_summary.xlsx
+++ b/publication/2026_07_10_results_xp_all_datasets_phd_contribution_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/399082/Documents/01_repositories/04_scMUG/publication/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8482CC18-50B6-FD4E-B1A6-7F5F11101E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5416E5B5-482C-7D48-9311-F2F7652EADE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{3E1E1FAC-2801-B847-9CD6-EE34F06970D1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{3E1E1FAC-2801-B847-9CD6-EE34F06970D1}"/>
   </bookViews>
   <sheets>
     <sheet name="ARI" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="32">
   <si>
     <t>Baron</t>
   </si>
@@ -287,7 +287,7 @@
         <rFont val="Helvetica Neue"/>
         <family val="2"/>
       </rPr>
-      <t>scDMKCN</t>
+      <t>Plugin</t>
     </r>
     <r>
       <rPr>
@@ -300,6 +300,39 @@
     </r>
     <r>
       <rPr>
+        <sz val="14"/>
+        <color theme="1" tint="0.499984740745262"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>(run Zeus 7 juill - 5 seeds)</t>
+    </r>
+  </si>
+  <si>
+    <t>Bloc A + Bloc B DMKCN + clust. EL</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>multikernel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
         <b/>
         <sz val="14"/>
         <color theme="1"/>
@@ -327,7 +360,7 @@
         <rFont val="Helvetica Neue"/>
         <family val="2"/>
       </rPr>
-      <t>scDMKCN</t>
+      <t>multi-kernel</t>
     </r>
     <r>
       <rPr>
@@ -356,36 +389,6 @@
         <family val="2"/>
       </rPr>
       <t>(locale - 5 seeds)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Helvetica Neue"/>
-        <family val="2"/>
-      </rPr>
-      <t>Plugin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Helvetica Neue"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1" tint="0.499984740745262"/>
-        <rFont val="Helvetica Neue"/>
-        <family val="2"/>
-      </rPr>
-      <t>(run Zeus 7 juill - 5 seeds)</t>
     </r>
   </si>
 </sst>
@@ -640,7 +643,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -651,26 +653,27 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -695,83 +698,121 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -805,107 +846,223 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1037,317 +1194,163 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1460,7 +1463,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <name val="Helvetica Neue"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -1499,63 +1502,63 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D19332C-9E1C-C64E-8289-AD00F630E34A}" name="Table1" displayName="Table1" ref="A1:L6" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D19332C-9E1C-C64E-8289-AD00F630E34A}" name="Table1" displayName="Table1" ref="A1:L6" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:L6" xr:uid="{6D19332C-9E1C-C64E-8289-AD00F630E34A}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{4A961F2C-C7B8-BA41-B501-A253E664E01E}" name="Dataset" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{03EEEB4F-9D7A-374B-BA8D-B82C799B65DD}" name="Genes" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{95CC7C03-1498-6B46-9946-28129E85C71C}" name="Cells" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{84FD71DF-EFDC-D042-A760-3BCD9C731443}" name="Labels" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{8F8830DD-B00E-5E46-8735-40DB5A10D137}" name="alpha/beta" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{29A6D3C2-8464-7640-8E5D-F218E0762B13}" name="scMUG (published)" dataDxfId="34"/>
-    <tableColumn id="11" xr3:uid="{50B50E3D-C90C-7545-B7E0-18632C029768}" name="scMUG (internal)" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{EABD17D8-7B9D-B044-8493-7A0D0465B069}" name="scDMKCN (published)" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{681A133D-C5EC-964A-8E61-6E323C42A2EA}" name="scDMKCN (internal)" dataDxfId="31"/>
-    <tableColumn id="12" xr3:uid="{FD91F65E-70DE-1F4B-B4A1-56C12FDF8EB2}" name="Plugin (internal)" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{AB942D1C-73BE-CF42-BE70-FC7C277C0D08}" name="Seurat" dataDxfId="29"/>
-    <tableColumn id="9" xr3:uid="{6E4A6D47-36E8-7B40-9BDA-19ABAACE2280}" name="Scanpy" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{4A961F2C-C7B8-BA41-B501-A253E664E01E}" name="Dataset" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{03EEEB4F-9D7A-374B-BA8D-B82C799B65DD}" name="Genes" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{95CC7C03-1498-6B46-9946-28129E85C71C}" name="Cells" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{84FD71DF-EFDC-D042-A760-3BCD9C731443}" name="Labels" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{8F8830DD-B00E-5E46-8735-40DB5A10D137}" name="alpha/beta" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{29A6D3C2-8464-7640-8E5D-F218E0762B13}" name="scMUG (published)" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{50B50E3D-C90C-7545-B7E0-18632C029768}" name="scMUG (internal)" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{EABD17D8-7B9D-B044-8493-7A0D0465B069}" name="scDMKCN (published)" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{681A133D-C5EC-964A-8E61-6E323C42A2EA}" name="scDMKCN (internal)" dataDxfId="17"/>
+    <tableColumn id="12" xr3:uid="{FD91F65E-70DE-1F4B-B4A1-56C12FDF8EB2}" name="Plugin (internal)" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{AB942D1C-73BE-CF42-BE70-FC7C277C0D08}" name="Seurat" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{6E4A6D47-36E8-7B40-9BDA-19ABAACE2280}" name="Scanpy" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D9DDC59-43EB-7449-8F66-B4EF7EA8735E}" name="Table15" displayName="Table15" ref="A1:L6" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D9DDC59-43EB-7449-8F66-B4EF7EA8735E}" name="Table15" displayName="Table15" ref="A1:L6" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="A1:L6" xr:uid="{6D19332C-9E1C-C64E-8289-AD00F630E34A}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{A2EA0FBC-D9EA-F64D-93ED-CFC0FE475D0A}" name="Dataset" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{C5D67021-4417-1846-AFDC-C6EA632B930F}" name="Genes" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{5FA0BD80-E44A-A946-8C06-B11FEBD2E782}" name="Cells" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{3B887553-94D0-1143-9487-F988A60CF74F}" name="Labels" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{7132453B-E973-B24D-B61B-CCFD321DA3B2}" name="alpha/beta" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{F868A95A-4F2E-DC47-9AAB-C2AD9361B9E4}" name="scMUG (published)" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{E525B1CA-0CF1-D544-90BA-39449E96E651}" name="scMUG (internal)" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{06789959-2FAC-BA42-97CE-CD497F78E81C}" name="scDMKCN (published)" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{984E7C23-A70B-3649-A562-E13BD4CBF425}" name="scDMKCN (internal)" dataDxfId="0"/>
-    <tableColumn id="12" xr3:uid="{1DEFCE9A-46B0-854E-8396-B90FCD0B1791}" name="Plugin (internal)" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{4B004D50-92AE-724C-8911-CD55D06B03B1}" name="Seurat" dataDxfId="21"/>
-    <tableColumn id="9" xr3:uid="{56E01CC7-392C-6B4F-B5A2-CDFEE0EAB77C}" name="Scanpy" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{A2EA0FBC-D9EA-F64D-93ED-CFC0FE475D0A}" name="Dataset" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{C5D67021-4417-1846-AFDC-C6EA632B930F}" name="Genes" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{5FA0BD80-E44A-A946-8C06-B11FEBD2E782}" name="Cells" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{3B887553-94D0-1143-9487-F988A60CF74F}" name="Labels" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{7132453B-E973-B24D-B61B-CCFD321DA3B2}" name="alpha/beta" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{F868A95A-4F2E-DC47-9AAB-C2AD9361B9E4}" name="scMUG (published)" dataDxfId="34"/>
+    <tableColumn id="11" xr3:uid="{E525B1CA-0CF1-D544-90BA-39449E96E651}" name="scMUG (internal)" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{06789959-2FAC-BA42-97CE-CD497F78E81C}" name="scDMKCN (published)" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{984E7C23-A70B-3649-A562-E13BD4CBF425}" name="scDMKCN (internal)" dataDxfId="31"/>
+    <tableColumn id="12" xr3:uid="{1DEFCE9A-46B0-854E-8396-B90FCD0B1791}" name="Plugin (internal)" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{4B004D50-92AE-724C-8911-CD55D06B03B1}" name="Seurat" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{56E01CC7-392C-6B4F-B5A2-CDFEE0EAB77C}" name="Scanpy" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{690A1E7C-4361-4342-BA40-1C6C8F82E91F}" name="Table156" displayName="Table156" ref="A1:L6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{690A1E7C-4361-4342-BA40-1C6C8F82E91F}" name="Table156" displayName="Table156" ref="A1:L6" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:L6" xr:uid="{6D19332C-9E1C-C64E-8289-AD00F630E34A}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{69DF850C-AF37-FF4E-B592-391A1B7F677B}" name="Dataset" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{FEB056B1-9F9D-BD4F-9835-E24DF324A190}" name="Genes" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{4A469DB2-5459-F442-BED4-A405B43277D8}" name="Cells" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{C45C4FE0-C9C5-7F49-A712-D9D572734984}" name="Labels" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{6CFDADBD-08E8-4746-A336-E3CD83D6722A}" name="alpha/beta" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{C93F801B-923F-E147-ABF4-F89D6B23117F}" name="scMUG (published)" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{ABD98428-AD6F-284E-8F9A-0BABA8494399}" name="scMUG (internal)" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{1835FC08-70DF-E74A-96B2-A483F7A0DCDD}" name="scDMKCN (published)" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{240C8A9E-CDA6-7F4E-A1D6-64D1F997A50E}" name="scDMKCN (internal)" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{5CFB3E25-12EE-244A-9754-C95F0483C49C}" name="Plugin (internal)" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{BDED31D3-0C20-9E4E-9CF4-A24B6D23AD80}" name="Seurat" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{83D2BA29-2DED-D74D-BBA9-445634BB5DD9}" name="Scanpy" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{69DF850C-AF37-FF4E-B592-391A1B7F677B}" name="Dataset" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{FEB056B1-9F9D-BD4F-9835-E24DF324A190}" name="Genes" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{4A469DB2-5459-F442-BED4-A405B43277D8}" name="Cells" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{C45C4FE0-C9C5-7F49-A712-D9D572734984}" name="Labels" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{6CFDADBD-08E8-4746-A336-E3CD83D6722A}" name="alpha/beta" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{C93F801B-923F-E147-ABF4-F89D6B23117F}" name="scMUG (published)" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{ABD98428-AD6F-284E-8F9A-0BABA8494399}" name="scMUG (internal)" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{1835FC08-70DF-E74A-96B2-A483F7A0DCDD}" name="scDMKCN (published)" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{240C8A9E-CDA6-7F4E-A1D6-64D1F997A50E}" name="scDMKCN (internal)" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{5CFB3E25-12EE-244A-9754-C95F0483C49C}" name="Plugin (internal)" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{BDED31D3-0C20-9E4E-9CF4-A24B6D23AD80}" name="Seurat" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{83D2BA29-2DED-D74D-BBA9-445634BB5DD9}" name="Scanpy" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2122,7 +2125,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3276987A-B0FF-5649-90FA-77A06BB2540F}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
@@ -2130,7 +2133,8 @@
     <col min="3" max="3" width="11" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="44.6640625" style="1" customWidth="1"/>
-    <col min="6" max="8" width="16.83203125" style="9" customWidth="1"/>
+    <col min="6" max="7" width="25.5" style="9" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" style="9" customWidth="1"/>
     <col min="9" max="9" width="26" style="9" customWidth="1"/>
     <col min="10" max="10" width="23.33203125" style="1" customWidth="1"/>
     <col min="11" max="12" width="13.6640625" style="1" customWidth="1"/>
@@ -2354,16 +2358,16 @@
     </row>
     <row r="14" spans="1:12" ht="19" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:12" ht="19" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="15" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2371,70 +2375,84 @@
       <c r="E16" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="F16" s="17">
+      <c r="F16" s="16">
         <v>0.91900000000000004</v>
       </c>
-      <c r="G16" s="17">
+      <c r="G16" s="16">
         <v>0.876</v>
       </c>
-      <c r="H16" s="18">
+      <c r="H16" s="17">
         <v>0.94699999999999995</v>
       </c>
     </row>
     <row r="17" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="18">
         <v>0.90659999999999996</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="18">
         <v>0.87119999999999997</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="19">
         <v>0.93759999999999999</v>
       </c>
     </row>
     <row r="18" spans="5:8" x14ac:dyDescent="0.2">
       <c r="E18" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="17">
+        <v>30</v>
+      </c>
+      <c r="F18" s="16">
         <v>0.91820000000000002</v>
       </c>
-      <c r="G18" s="17">
+      <c r="G18" s="16">
         <v>0.87749999999999995</v>
       </c>
-      <c r="H18" s="24" t="s">
+      <c r="H18" s="21" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E19" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="19">
+      <c r="E19" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="18">
         <v>0.88900000000000001</v>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="18">
         <v>0.84</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="19">
         <v>0.90200000000000002</v>
       </c>
     </row>
     <row r="20" spans="5:8" ht="19" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E20" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F20" s="21">
+      <c r="E20" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="23">
         <v>0.9073</v>
       </c>
-      <c r="G20" s="21">
+      <c r="G20" s="23">
         <v>0.86860000000000004</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="24">
         <v>0.95189999999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="6">
+        <v>0.87760000000000005</v>
+      </c>
+      <c r="G21" s="6">
+        <v>0.82909999999999995</v>
+      </c>
+      <c r="H21" s="6">
+        <v>0.89180000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>